<commit_message>
Add SVG QR exports
</commit_message>
<xml_diff>
--- a/input/Sample.xlsx
+++ b/input/Sample.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$2:$X$129</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$2:$X$130</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -15202,6 +15202,7 @@
       <c r="R127" t="n">
         <v>78</v>
       </c>
+      <c r="S127" t="inlineStr"/>
       <c r="W127" t="inlineStr">
         <is>
           <t>640</t>
@@ -15318,6 +15319,7 @@
       <c r="R128" t="n">
         <v>56</v>
       </c>
+      <c r="S128" t="inlineStr"/>
       <c r="W128" t="inlineStr">
         <is>
           <t>640</t>
@@ -15434,6 +15436,7 @@
       <c r="R129" t="n">
         <v>90</v>
       </c>
+      <c r="S129" t="inlineStr"/>
       <c r="W129" t="inlineStr">
         <is>
           <t>640</t>
@@ -15504,10 +15507,8 @@
           <t>80</t>
         </is>
       </c>
-      <c r="I130" t="inlineStr">
-        <is>
-          <t>56</t>
-        </is>
+      <c r="I130" t="n">
+        <v>56</v>
       </c>
       <c r="J130" t="inlineStr">
         <is>
@@ -15553,9 +15554,6 @@
         <v>70</v>
       </c>
       <c r="S130" t="inlineStr"/>
-      <c r="T130" t="inlineStr"/>
-      <c r="U130" t="inlineStr"/>
-      <c r="V130" t="inlineStr"/>
       <c r="W130" t="inlineStr">
         <is>
           <t>Unit 1</t>
@@ -15588,42 +15586,42 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:X129"/>
+  <autoFilter ref="A2:X130"/>
   <dataValidations count="12">
-    <dataValidation sqref="D3:D129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="D3:D130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Trg,Svl (SR),Svl (MR),FPV,Kamikaze,Lgs,Loitering Munition"</formula1>
     </dataValidation>
-    <dataValidation sqref="E3:E129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E3:E130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"QC,HC,Fixed Wg,FIxed Wing VTOL,Swarm"</formula1>
     </dataValidation>
-    <dataValidation sqref="G3:G129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G3:G130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"&lt; 5 km,5-10 km,10-30 km,31-100 km,&gt; 100 km"</formula1>
     </dataValidation>
-    <dataValidation sqref="O3:O129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="O3:O130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"1.4 GHz,2.4 GHz,5.8 GHz,900 MHz"</formula1>
     </dataValidation>
-    <dataValidation sqref="P3:P129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="P3:P130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"ATG,Regtl,Unit,Central"</formula1>
     </dataValidation>
-    <dataValidation sqref="Q3:Q129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="Q3:Q130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Ser,Unser"</formula1>
     </dataValidation>
-    <dataValidation sqref="F3:F129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F3:F130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Northern Security Pvt Ltd,OEM Alpha,OEM Bravo,OEM Delta,OEM Kilo,OEM Nova,OEM Zenith,oem c"</formula1>
     </dataValidation>
-    <dataValidation sqref="W3:W129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="W3:W130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"640,640EME,Unit 1,Unit 10,Unit 11,Unit 12,Unit 2,Unit 3,Unit 4,Unit 5,Unit 6,Unit 7,Unit 8,Unit 9"</formula1>
     </dataValidation>
-    <dataValidation sqref="X3:X129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="X3:X130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"371B,40D,Brigade 1,Brigade 2,Brigade 3,Brigade 4,Brigade 5,Brigade 6,New Brigade"</formula1>
     </dataValidation>
-    <dataValidation sqref="Y3:Y129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="Y3:Y130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"40D,Division Alpha,New Division"</formula1>
     </dataValidation>
-    <dataValidation sqref="Z3:Z129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="Z3:Z130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"2C,Corps North,New Corps"</formula1>
     </dataValidation>
-    <dataValidation sqref="AA3:AA129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="AA3:AA130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Command East,New Command,WC,cc"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Remove legacy UID workflow and dummy data
</commit_message>
<xml_diff>
--- a/input/Sample.xlsx
+++ b/input/Sample.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$2:$X$130</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$2:$AB$1002</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,13 +27,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -48,8 +62,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -449,192 +467,174 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Drone Inventory - Schema Migrated</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Drone Inventory - KUIN-G Input</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Ser No</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Drone ID</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Drone Name</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Form Factor</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>OEM</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Range</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Weight (KG)</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Endurance (min)</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Payload</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Payload Weight</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Payload Description</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Guidance</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Anti Ew</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>C2 Link Frequency</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>Proc Fund</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>Serv</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>Cost (in Thousands)</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="S2" s="2" t="inlineStr">
         <is>
           <t>Image Front</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="T2" s="2" t="inlineStr">
         <is>
           <t>Image Back</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="U2" s="2" t="inlineStr">
         <is>
           <t>Image Top</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="V2" s="2" t="inlineStr">
         <is>
           <t>Image Bottom</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="W2" s="2" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="X2" s="2" t="inlineStr">
         <is>
           <t>Brigade</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="Y2" s="2" t="inlineStr">
         <is>
           <t>Division</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="Z2" s="2" t="inlineStr">
         <is>
           <t>Corps</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AA2" s="2" t="inlineStr">
         <is>
           <t>Command</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AB2" s="2" t="inlineStr">
         <is>
           <t>KUIN-G</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:X130"/>
-  <dataValidations count="12">
-    <dataValidation sqref="D3:D130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+  <autoFilter ref="A2:AB1002"/>
+  <dataValidations count="6">
+    <dataValidation sqref="D3:D1002" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Trg,Svl (SR),Svl (MR),FPV,Kamikaze,Lgs,Loitering Munition"</formula1>
     </dataValidation>
-    <dataValidation sqref="E3:E130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E3:E1002" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"QC,HC,Fixed Wg,FIxed Wing VTOL,Swarm"</formula1>
     </dataValidation>
-    <dataValidation sqref="G3:G130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G3:G1002" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"&lt; 5 km,5-10 km,10-30 km,31-100 km,&gt; 100 km"</formula1>
     </dataValidation>
-    <dataValidation sqref="O3:O130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="O3:O1002" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"1.4 GHz,2.4 GHz,5.8 GHz,900 MHz"</formula1>
     </dataValidation>
-    <dataValidation sqref="P3:P130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="P3:P1002" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"ATG,Regtl,Unit,Central"</formula1>
     </dataValidation>
-    <dataValidation sqref="Q3:Q130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="Q3:Q1002" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Ser,Unser"</formula1>
-    </dataValidation>
-    <dataValidation sqref="F3:F130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Northern Security Pvt Ltd,OEM Alpha,OEM Bravo,OEM Delta,OEM Kilo,OEM Nova,OEM Zenith,oem c"</formula1>
-    </dataValidation>
-    <dataValidation sqref="W3:W130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"640,640EME,Unit 1,Unit 10,Unit 11,Unit 12,Unit 2,Unit 3,Unit 4,Unit 5,Unit 6,Unit 7,Unit 8,Unit 9"</formula1>
-    </dataValidation>
-    <dataValidation sqref="X3:X130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"371B,40D,Brigade 1,Brigade 2,Brigade 3,Brigade 4,Brigade 5,Brigade 6,New Brigade"</formula1>
-    </dataValidation>
-    <dataValidation sqref="Y3:Y130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"40D,Division Alpha,New Division"</formula1>
-    </dataValidation>
-    <dataValidation sqref="Z3:Z130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"2C,Corps North,New Corps"</formula1>
-    </dataValidation>
-    <dataValidation sqref="AA3:AA130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Command East,New Command,WC,cc"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Include current KUIN-G database and QR data
</commit_message>
<xml_diff>
--- a/input/Sample.xlsx
+++ b/input/Sample.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:AB10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -615,6 +615,931 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>WC-2C-40A-000X-640E-ANA-SVL-01</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Anant Drishti</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Svl</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Hexacopter</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Marsaero Innovations</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>&lt; 5 km</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>480</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>EO IR Camera</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>30x Digital zoom</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Tethered with GPS</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Tethered with EW Resilience</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Nil</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>SRE</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Ser</t>
+        </is>
+      </c>
+      <c r="R3" t="n">
+        <v>1100</v>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>640 EME Bn</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>000</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>40 Arty Div</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>2 Corps</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>WC</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>DDD52MN3XCB6YBD7</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>WC-2C-40A-000X-640E-ANV-SVL-02</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Anveshak v1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Svl</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Quadcopter</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Northern Security</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>&lt; 5 km</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Day Ni Camera</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>GNSS</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Nil</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>1.4 GHz</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>ACG</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Ser</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>640 EME Bn</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>000</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>40 Arty Div</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>2 Corps</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>WC</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>JBOA6DY5HEVS5VAE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>WC-2C-40A-000X-640E-ANV-SVL-03</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Anveshak v1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Svl</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Quadcopter</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Northern Security</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>&lt; 5 km</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Day Ni Camera</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>GNSS</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Nil</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>1.4 GHz</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>ACG</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Ser</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>640 EME Bn</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>000</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>40 Arty Div</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>2 Corps</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>WC</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>VI5NAR2U7UJUQ75P</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>WC-2C-40A-000X-640E-ANV-SVL-04</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anveshak V1 </t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Svl</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Quadcopter</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Northern Security</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>&lt; 5 km</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Day Ni Camera</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>GNSS</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Nil</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>1.4 GHz</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>ACG</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Ser</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>297</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>640 EME Bn</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>000</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>40 Arty Div</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>2 Corps</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>WC</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>G7KKZQVFT5RSEXLS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>WC-2C-40A-000X-640E-KHA-LMX-05</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Kharga Chakra</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>LM</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>VTOL</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Xagrotor</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>&gt; 100 km</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>240</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Munition; EO IR Camera</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>3; 2</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Upto 5 kg without camera; total 5 kg</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>GNSS</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>4 Element CRPA</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>2.4-5.8 GHz</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>IR&amp;D</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Unser</t>
+        </is>
+      </c>
+      <c r="R7" t="n">
+        <v>7400</v>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>640 EME Bn</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>000</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>40 Arty Div</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>2 Corps</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>WC</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>CCX2QDL6IJJ3SCRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>WC-2C-40A-000X-640E-20K-SVL-06</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>20 Km Fixed wing Svl Drone</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Svl</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>VTOL</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Northern Security</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>10-30 km</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>EO IR Camera</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>GNSS</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Nil</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>2.4-5.8 GHz</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>TTIEG</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Ser</t>
+        </is>
+      </c>
+      <c r="R8" t="n">
+        <v>0</v>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>640 EME Bn</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>000</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>40 Arty Div</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>2 Corps</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>WC</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>EVNPVZZ4PINRHY3A</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>WC-2C-40A-000X-640E-ANV-SVL-07</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Anveshak V2</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Svl</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Quadcopter</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Marsaero Innovations</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>5-10 km</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Day Ni Camera</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>GNSS</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>FHSS Dual band</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>2.4-5.8 GHz</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>IR&amp;D</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Ser</t>
+        </is>
+      </c>
+      <c r="R9" t="n">
+        <v>647</v>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>640 EME Bn</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>000</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>40 Arty Div</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>2 Corps</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>WC</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>B5J6XXJHV3RQQQWH</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>WC-2C-40A-000X-640E-8BI-SWA-08</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>8 Bird Svl Swarm Drone</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Swarm Drone- Svl</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Quadcopter</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Xagrotor</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>10-30 km</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>EO IR Camera</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>GNSS</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Nil</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>2.4-5.8 GHz</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>IR&amp;D</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Ser</t>
+        </is>
+      </c>
+      <c r="R10" t="n">
+        <v>19800</v>
+      </c>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>640 EME Bn</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>000</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>40 Arty Div</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>2 Corps</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>WC</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>5LEPA4HRFWDM47M4</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A2:AB1002"/>
   <dataValidations count="6">

</xml_diff>

<commit_message>
Update drone register schema and dashboard
</commit_message>
<xml_diff>
--- a/input/Sample.xlsx
+++ b/input/Sample.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$2:$AB$1002</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$2:$AC$1002</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB10"/>
+  <dimension ref="A1:AC10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -521,95 +521,100 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
+          <t>Day/Night Capability</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
           <t>Payload</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Payload Weight</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Payload Description</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Guidance</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>Anti Ew</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>C2 Link Frequency</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>Proc Fund</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr">
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>Serv</t>
         </is>
       </c>
-      <c r="R2" s="2" t="inlineStr">
+      <c r="S2" s="2" t="inlineStr">
         <is>
           <t>Cost (in Thousands)</t>
         </is>
       </c>
-      <c r="S2" s="2" t="inlineStr">
+      <c r="T2" s="2" t="inlineStr">
         <is>
           <t>Image Front</t>
         </is>
       </c>
-      <c r="T2" s="2" t="inlineStr">
+      <c r="U2" s="2" t="inlineStr">
         <is>
           <t>Image Back</t>
         </is>
       </c>
-      <c r="U2" s="2" t="inlineStr">
+      <c r="V2" s="2" t="inlineStr">
         <is>
           <t>Image Top</t>
         </is>
       </c>
-      <c r="V2" s="2" t="inlineStr">
+      <c r="W2" s="2" t="inlineStr">
         <is>
           <t>Image Bottom</t>
         </is>
       </c>
-      <c r="W2" s="2" t="inlineStr">
+      <c r="X2" s="2" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="X2" s="2" t="inlineStr">
+      <c r="Y2" s="2" t="inlineStr">
         <is>
           <t>Brigade</t>
         </is>
       </c>
-      <c r="Y2" s="2" t="inlineStr">
+      <c r="Z2" s="2" t="inlineStr">
         <is>
           <t>Division</t>
         </is>
       </c>
-      <c r="Z2" s="2" t="inlineStr">
+      <c r="AA2" s="2" t="inlineStr">
         <is>
           <t>Corps</t>
         </is>
       </c>
-      <c r="AA2" s="2" t="inlineStr">
+      <c r="AB2" s="2" t="inlineStr">
         <is>
           <t>Command</t>
         </is>
       </c>
-      <c r="AB2" s="2" t="inlineStr">
+      <c r="AC2" s="2" t="inlineStr">
         <is>
           <t>KUIN-G</t>
         </is>
@@ -659,75 +664,75 @@
           <t>480</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>EO IR Camera</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>0.8</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>30x Digital zoom</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Tethered with GPS</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>Tethered with EW Resilience</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>Nil</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>SRE</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>Ser</t>
         </is>
       </c>
-      <c r="R3" t="n">
+      <c r="S3" t="n">
         <v>1100</v>
       </c>
-      <c r="W3" t="inlineStr">
+      <c r="X3" t="inlineStr">
         <is>
           <t>640 EME Bn</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="Y3" t="inlineStr">
         <is>
           <t>000</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr">
+      <c r="Z3" t="inlineStr">
         <is>
           <t>40 Arty Div</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
+      <c r="AA3" t="inlineStr">
         <is>
           <t>2 Corps</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr">
+      <c r="AB3" t="inlineStr">
         <is>
           <t>WC</t>
         </is>
       </c>
-      <c r="AB3" t="inlineStr">
+      <c r="AC3" t="inlineStr">
         <is>
           <t>DDD52MN3XCB6YBD7</t>
         </is>
@@ -777,72 +782,72 @@
           <t>30</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Day Ni Camera</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>0.3</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>GNSS</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>Nil</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>1.4 GHz</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>ACG</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>Ser</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>300</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="X4" t="inlineStr">
         <is>
           <t>640 EME Bn</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>000</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr">
+      <c r="Z4" t="inlineStr">
         <is>
           <t>40 Arty Div</t>
         </is>
       </c>
-      <c r="Z4" t="inlineStr">
+      <c r="AA4" t="inlineStr">
         <is>
           <t>2 Corps</t>
         </is>
       </c>
-      <c r="AA4" t="inlineStr">
+      <c r="AB4" t="inlineStr">
         <is>
           <t>WC</t>
         </is>
       </c>
-      <c r="AB4" t="inlineStr">
+      <c r="AC4" t="inlineStr">
         <is>
           <t>JBOA6DY5HEVS5VAE</t>
         </is>
@@ -892,72 +897,72 @@
           <t>30</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Day Ni Camera</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>0.3</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>GNSS</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>Nil</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>1.4 GHz</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>ACG</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>Ser</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>300</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr">
+      <c r="X5" t="inlineStr">
         <is>
           <t>640 EME Bn</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr">
+      <c r="Y5" t="inlineStr">
         <is>
           <t>000</t>
         </is>
       </c>
-      <c r="Y5" t="inlineStr">
+      <c r="Z5" t="inlineStr">
         <is>
           <t>40 Arty Div</t>
         </is>
       </c>
-      <c r="Z5" t="inlineStr">
+      <c r="AA5" t="inlineStr">
         <is>
           <t>2 Corps</t>
         </is>
       </c>
-      <c r="AA5" t="inlineStr">
+      <c r="AB5" t="inlineStr">
         <is>
           <t>WC</t>
         </is>
       </c>
-      <c r="AB5" t="inlineStr">
+      <c r="AC5" t="inlineStr">
         <is>
           <t>VI5NAR2U7UJUQ75P</t>
         </is>
@@ -1007,72 +1012,72 @@
           <t>30</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>Day Ni Camera</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>0.3</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>GNSS</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>Nil</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>1.4 GHz</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>ACG</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t>Ser</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>297</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr">
+      <c r="X6" t="inlineStr">
         <is>
           <t>640 EME Bn</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr">
+      <c r="Y6" t="inlineStr">
         <is>
           <t>000</t>
         </is>
       </c>
-      <c r="Y6" t="inlineStr">
+      <c r="Z6" t="inlineStr">
         <is>
           <t>40 Arty Div</t>
         </is>
       </c>
-      <c r="Z6" t="inlineStr">
+      <c r="AA6" t="inlineStr">
         <is>
           <t>2 Corps</t>
         </is>
       </c>
-      <c r="AA6" t="inlineStr">
+      <c r="AB6" t="inlineStr">
         <is>
           <t>WC</t>
         </is>
       </c>
-      <c r="AB6" t="inlineStr">
+      <c r="AC6" t="inlineStr">
         <is>
           <t>G7KKZQVFT5RSEXLS</t>
         </is>
@@ -1122,75 +1127,75 @@
           <t>240</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>Munition; EO IR Camera</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>3; 2</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>Upto 5 kg without camera; total 5 kg</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>GNSS</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>4 Element CRPA</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>2.4-5.8 GHz</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>IR&amp;D</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="R7" t="inlineStr">
         <is>
           <t>Unser</t>
         </is>
       </c>
-      <c r="R7" t="n">
+      <c r="S7" t="n">
         <v>7400</v>
       </c>
-      <c r="W7" t="inlineStr">
+      <c r="X7" t="inlineStr">
         <is>
           <t>640 EME Bn</t>
         </is>
       </c>
-      <c r="X7" t="inlineStr">
+      <c r="Y7" t="inlineStr">
         <is>
           <t>000</t>
         </is>
       </c>
-      <c r="Y7" t="inlineStr">
+      <c r="Z7" t="inlineStr">
         <is>
           <t>40 Arty Div</t>
         </is>
       </c>
-      <c r="Z7" t="inlineStr">
+      <c r="AA7" t="inlineStr">
         <is>
           <t>2 Corps</t>
         </is>
       </c>
-      <c r="AA7" t="inlineStr">
+      <c r="AB7" t="inlineStr">
         <is>
           <t>WC</t>
         </is>
       </c>
-      <c r="AB7" t="inlineStr">
+      <c r="AC7" t="inlineStr">
         <is>
           <t>CCX2QDL6IJJ3SCRA</t>
         </is>
@@ -1240,70 +1245,70 @@
           <t>90</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>EO IR Camera</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>GNSS</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>Nil</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>2.4-5.8 GHz</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>TTIEG</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr">
+      <c r="R8" t="inlineStr">
         <is>
           <t>Ser</t>
         </is>
       </c>
-      <c r="R8" t="n">
+      <c r="S8" t="n">
         <v>0</v>
       </c>
-      <c r="W8" t="inlineStr">
+      <c r="X8" t="inlineStr">
         <is>
           <t>640 EME Bn</t>
         </is>
       </c>
-      <c r="X8" t="inlineStr">
+      <c r="Y8" t="inlineStr">
         <is>
           <t>000</t>
         </is>
       </c>
-      <c r="Y8" t="inlineStr">
+      <c r="Z8" t="inlineStr">
         <is>
           <t>40 Arty Div</t>
         </is>
       </c>
-      <c r="Z8" t="inlineStr">
+      <c r="AA8" t="inlineStr">
         <is>
           <t>2 Corps</t>
         </is>
       </c>
-      <c r="AA8" t="inlineStr">
+      <c r="AB8" t="inlineStr">
         <is>
           <t>WC</t>
         </is>
       </c>
-      <c r="AB8" t="inlineStr">
+      <c r="AC8" t="inlineStr">
         <is>
           <t>EVNPVZZ4PINRHY3A</t>
         </is>
@@ -1353,70 +1358,70 @@
           <t>30</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>Day Ni Camera</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>0.3</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>GNSS</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>FHSS Dual band</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>2.4-5.8 GHz</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>IR&amp;D</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr">
+      <c r="R9" t="inlineStr">
         <is>
           <t>Ser</t>
         </is>
       </c>
-      <c r="R9" t="n">
+      <c r="S9" t="n">
         <v>647</v>
       </c>
-      <c r="W9" t="inlineStr">
+      <c r="X9" t="inlineStr">
         <is>
           <t>640 EME Bn</t>
         </is>
       </c>
-      <c r="X9" t="inlineStr">
+      <c r="Y9" t="inlineStr">
         <is>
           <t>000</t>
         </is>
       </c>
-      <c r="Y9" t="inlineStr">
+      <c r="Z9" t="inlineStr">
         <is>
           <t>40 Arty Div</t>
         </is>
       </c>
-      <c r="Z9" t="inlineStr">
+      <c r="AA9" t="inlineStr">
         <is>
           <t>2 Corps</t>
         </is>
       </c>
-      <c r="AA9" t="inlineStr">
+      <c r="AB9" t="inlineStr">
         <is>
           <t>WC</t>
         </is>
       </c>
-      <c r="AB9" t="inlineStr">
+      <c r="AC9" t="inlineStr">
         <is>
           <t>B5J6XXJHV3RQQQWH</t>
         </is>
@@ -1466,78 +1471,78 @@
           <t>65</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>EO IR Camera</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>GNSS</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>Nil</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>2.4-5.8 GHz</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="Q10" t="inlineStr">
         <is>
           <t>IR&amp;D</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr">
+      <c r="R10" t="inlineStr">
         <is>
           <t>Ser</t>
         </is>
       </c>
-      <c r="R10" t="n">
+      <c r="S10" t="n">
         <v>19800</v>
       </c>
-      <c r="W10" t="inlineStr">
+      <c r="X10" t="inlineStr">
         <is>
           <t>640 EME Bn</t>
         </is>
       </c>
-      <c r="X10" t="inlineStr">
+      <c r="Y10" t="inlineStr">
         <is>
           <t>000</t>
         </is>
       </c>
-      <c r="Y10" t="inlineStr">
+      <c r="Z10" t="inlineStr">
         <is>
           <t>40 Arty Div</t>
         </is>
       </c>
-      <c r="Z10" t="inlineStr">
+      <c r="AA10" t="inlineStr">
         <is>
           <t>2 Corps</t>
         </is>
       </c>
-      <c r="AA10" t="inlineStr">
+      <c r="AB10" t="inlineStr">
         <is>
           <t>WC</t>
         </is>
       </c>
-      <c r="AB10" t="inlineStr">
+      <c r="AC10" t="inlineStr">
         <is>
           <t>5LEPA4HRFWDM47M4</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AB1002"/>
-  <dataValidations count="6">
+  <autoFilter ref="A2:AC1002"/>
+  <dataValidations count="7">
     <dataValidation sqref="D3:D1002" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Trg,Svl (SR),Svl (MR),FPV,Kamikaze,Lgs,Loitering Munition"</formula1>
     </dataValidation>
@@ -1547,14 +1552,17 @@
     <dataValidation sqref="G3:G1002" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"&lt; 5 km,5-10 km,10-30 km,31-100 km,&gt; 100 km"</formula1>
     </dataValidation>
-    <dataValidation sqref="O3:O1002" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="P3:P1002" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"1.4 GHz,2.4 GHz,5.8 GHz,900 MHz"</formula1>
     </dataValidation>
-    <dataValidation sqref="P3:P1002" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="Q3:Q1002" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"ATG,Regtl,Unit,Central"</formula1>
     </dataValidation>
-    <dataValidation sqref="Q3:Q1002" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="R3:R1002" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Ser,Unser"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J3:J1002" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid value" error="Select Day or Night." type="list">
+      <formula1>"Day,Night"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>